<commit_message>
feat: update sales dashboard and synchronize data sources
Atualização do arquivo .pbix com a nova modelagem Star Schema.

Inclusão de novas bases de dados (clientes, vendas e vendedores) em formato Excel.

Ajuste de medidas DAX e formatação dinâmica de valores.
</commit_message>
<xml_diff>
--- a/SQL/PostgreSQL/Projeto Vendas/Dados/base_clientes.xlsx
+++ b/SQL/PostgreSQL/Projeto Vendas/Dados/base_clientes.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30006"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\waccache\CP1PEPF00001F18\EXCELCNV\9c2f98c3-b08e-4bfc-b2bb-097aa8bd332d\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\biblioteca\Projetos 2026\Estudos Iniciais\Estudo de dados\SQL\PostgreSQL\Projeto Vendas\Dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2C5A289-81C6-4DFF-8D50-658877FDEF6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" xr2:uid="{4873B5F0-4D92-4565-993C-B1CAF7632696}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12285"/>
   </bookViews>
   <sheets>
     <sheet name="in" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="85">
   <si>
     <t>id_cliente</t>
   </si>
@@ -90,13 +89,214 @@
   </si>
   <si>
     <t>Jihyo</t>
+  </si>
+  <si>
+    <t>Sasha Banks</t>
+  </si>
+  <si>
+    <t>Boston</t>
+  </si>
+  <si>
+    <t>Toni Storm</t>
+  </si>
+  <si>
+    <t>Auckland</t>
+  </si>
+  <si>
+    <t>Ronda Rousey</t>
+  </si>
+  <si>
+    <t>Riverside</t>
+  </si>
+  <si>
+    <t>Rhea Ripley</t>
+  </si>
+  <si>
+    <t>Adelaide</t>
+  </si>
+  <si>
+    <t>Becky Lynch</t>
+  </si>
+  <si>
+    <t>Dublin</t>
+  </si>
+  <si>
+    <t>Eimi Gloria Matsudo</t>
+  </si>
+  <si>
+    <t>Londres</t>
+  </si>
+  <si>
+    <t>Lyra Valkyria</t>
+  </si>
+  <si>
+    <t>Asuka</t>
+  </si>
+  <si>
+    <t>Osaka</t>
+  </si>
+  <si>
+    <t>Jade Cargill</t>
+  </si>
+  <si>
+    <t>Vero Beach</t>
+  </si>
+  <si>
+    <t>Tiffany Stratton</t>
+  </si>
+  <si>
+    <t>Prior Lake</t>
+  </si>
+  <si>
+    <t>Kim Minji</t>
+  </si>
+  <si>
+    <t>Chuncheon</t>
+  </si>
+  <si>
+    <t>Hanni Pham</t>
+  </si>
+  <si>
+    <t>Melbourne</t>
+  </si>
+  <si>
+    <t>Kang Haerin</t>
+  </si>
+  <si>
+    <t>Anyang</t>
+  </si>
+  <si>
+    <t>Hwang Yeji</t>
+  </si>
+  <si>
+    <t>Jeonju</t>
+  </si>
+  <si>
+    <t>Shin Ryujin</t>
+  </si>
+  <si>
+    <t>Lee Chaeryeong</t>
+  </si>
+  <si>
+    <t>Yongin</t>
+  </si>
+  <si>
+    <t>Momo Hirai</t>
+  </si>
+  <si>
+    <t>Quioto</t>
+  </si>
+  <si>
+    <t>Sana Minatozaki</t>
+  </si>
+  <si>
+    <t>Mina Myoi</t>
+  </si>
+  <si>
+    <t>San Antonio</t>
+  </si>
+  <si>
+    <t>Freen Sarocha</t>
+  </si>
+  <si>
+    <t>Bangkok</t>
+  </si>
+  <si>
+    <t>Ling Ling Kwong</t>
+  </si>
+  <si>
+    <t>Becky Armstrong</t>
+  </si>
+  <si>
+    <t>Orm Kornnaphat</t>
+  </si>
+  <si>
+    <t>Charlotte Austin</t>
+  </si>
+  <si>
+    <t>Phuket</t>
+  </si>
+  <si>
+    <t>Engfa Waraha</t>
+  </si>
+  <si>
+    <t>Uthai Thani</t>
+  </si>
+  <si>
+    <t>Milk Pansa</t>
+  </si>
+  <si>
+    <t>Love Pattranite</t>
+  </si>
+  <si>
+    <t>Faye Peraya</t>
+  </si>
+  <si>
+    <t>Yoko Apasra</t>
+  </si>
+  <si>
+    <t>Mai Shiranui</t>
+  </si>
+  <si>
+    <t>Tóquio</t>
+  </si>
+  <si>
+    <t>King</t>
+  </si>
+  <si>
+    <t>Paris</t>
+  </si>
+  <si>
+    <t>Blue Mary</t>
+  </si>
+  <si>
+    <t>Miami</t>
+  </si>
+  <si>
+    <t>Ling Xiaoyu</t>
+  </si>
+  <si>
+    <t>Pequim</t>
+  </si>
+  <si>
+    <t>Jun Kazama</t>
+  </si>
+  <si>
+    <t>Yakushima</t>
+  </si>
+  <si>
+    <t>Asuka Kazama</t>
+  </si>
+  <si>
+    <t>Nina Williams</t>
+  </si>
+  <si>
+    <t>Kitana</t>
+  </si>
+  <si>
+    <t>Mileena</t>
+  </si>
+  <si>
+    <t>Cairo</t>
+  </si>
+  <si>
+    <t>Jade</t>
+  </si>
+  <si>
+    <t>Brasília</t>
+  </si>
+  <si>
+    <t>Sonya Blade</t>
+  </si>
+  <si>
+    <t>Austin</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -573,11 +773,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" xfId="38" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" xfId="38"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -609,10 +810,10 @@
     <cellStyle name="Ênfase5" xfId="34" builtinId="45" customBuiltin="1"/>
     <cellStyle name="Ênfase6" xfId="38" builtinId="49" customBuiltin="1"/>
     <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Neutro" xfId="8" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="Incorreto" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Neutra" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Nota" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Ruim" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Saída" xfId="10" builtinId="21" customBuiltin="1"/>
     <cellStyle name="Texto de Aviso" xfId="14" builtinId="11" customBuiltin="1"/>
     <cellStyle name="Texto Explicativo" xfId="16" builtinId="53" customBuiltin="1"/>
@@ -639,7 +840,7 @@
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Escala de Cinza">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -647,34 +848,34 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="F8F8F8"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="DDDDDD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="B2B2B2"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="969696"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="808080"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="5F5F5F"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="4D4D4D"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="5F5F5F"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="919191"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -932,11 +1133,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60C6BF9F-804C-4892-8CD4-5365A154923B}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H50"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="2"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -947,7 +1154,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>2</v>
       </c>
@@ -958,7 +1165,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>3</v>
       </c>
@@ -969,7 +1176,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>4</v>
       </c>
@@ -980,7 +1187,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>5</v>
       </c>
@@ -991,7 +1198,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>6</v>
       </c>
@@ -1002,7 +1209,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>7</v>
       </c>
@@ -1013,7 +1220,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>8</v>
       </c>
@@ -1024,7 +1231,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>9</v>
       </c>
@@ -1035,7 +1242,462 @@
         <v>4</v>
       </c>
     </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>10</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>11</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>12</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>13</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>14</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>15</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>16</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>17</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>18</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>19</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>20</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>21</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>22</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>23</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>24</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>25</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>26</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>27</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>28</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>29</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>30</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>31</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>32</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>33</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>34</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>35</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>36</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>37</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>38</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>39</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>40</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>41</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>42</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>43</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
+        <v>44</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="1">
+        <v>45</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" s="1">
+        <v>46</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
+        <v>47</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" s="1">
+        <v>48</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
+        <v>49</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
+        <v>50</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>